<commit_message>
fix(scripts): close DB on import failure; update client needs sheet from legacy import
Import scripts left the MySQL pool open when they failed early (e.g.
missing KML), so the process hung instead of exiting. The needs sheet now
marks what the old site supplied and lists the questions left.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data/media-and-content-needs.xlsx
+++ b/docs/data/media-and-content-needs.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="What we need" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Samithi details" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What we need" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samithi details" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'What we need'!$A$1:$H$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Samithi details'!$A$1:$G$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'What we need'!$A$1:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Samithi details'!$A$1:$I$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -528,7 +528,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Go to 'What we need'. Set Status on each row. Row 7 points to the 'Samithi details' sheet.</t>
+          <t>Go to 'What we need'. Set Status on each row. Row 7 points to the 'Samithi details' sheet. Rows 8 to 14 were added on 28 Oct 2026.</t>
         </is>
       </c>
     </row>
@@ -585,6 +585,13 @@
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>If rights are unclear, send it anyway and mark it 'rights unknown'. We will not publish it until cleared.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Samithi details: please also give weekly gathering times and a phone number we may show publicly (columns H and I).</t>
         </is>
       </c>
     </row>
@@ -599,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -685,10 +692,14 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Using about 10 photos from the old website (540 to 860 px). Please send larger originals (2000 px or more) if you have them.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -721,10 +732,14 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Have the International Centre and auditorium from the old website. Still need photos of other centres.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -757,10 +772,14 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr"/>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>444 photos taken from the old website news posts. New photos welcome any time.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -793,10 +812,14 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr"/>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Taken from the old website.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -829,10 +852,14 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>ICARE logo can be taken from its website. Others depend on the partner list (row 12).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -853,7 +880,7 @@
           <t>1. Official WhatsApp number to publish.
 2. Access to the WhatsApp Business / Meta account (by phone call only, not chat).
 3. About page text: contact details, auditorium details, founder section.
-4. Written permission from Sadhana Trust to publish the discourses.
+4. Written permission from Sadhana Trust to publish the discourses and the daily Thought for the Day.
 5. Name of the data-protection contact.
 6. Samithi details: local name, address and Google Maps pin for each samithi (use the "Samithi details" sheet).</t>
         </is>
@@ -870,15 +897,299 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Have from the old website: WhatsApp number +91 99719 99991, About text, samithi map pins and area names. Still need: Meta/WhatsApp Business access (by phone), data-protection contact name, Sadhana Trust permission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Donation bank details (confirm)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>The Donate page shows the Sri Sathya Sai Trust, Delhi &amp; Punjab bank account taken from the old website: account name, bank, branch, account number, IFSC, MICR, and the email for receipts and 80G certificates (sp.dl@ssssoindia.org). Please confirm every value is still correct.</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Scanned letter or email from the Trust treasurer confirming the details.</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Written confirmation from the Trust. We will not publish bank details without it.</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Taken from the old website Get Involved page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>First portal administrators</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Name and WhatsApp number of 1 or 2 state-level people who will run the coordinator portal. They then invite district and samithi coordinators from inside the portal.</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Name, role and WhatsApp number. By phone call or in person.</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>The person agrees to be an administrator. Numbers are not shown publicly.</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Office bearers and samithi conveners taken from the old website and invited to the portal. Question: Gurugram and West each list two different District Presidents. Who is current?</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Contact details to confirm</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>1. State office phone, email and postal address (About page).
+2. International Centre, Lodhi Road: phones 011-2436 3221 and 011-2436 0190, hours "all days 10 AM to 6 PM", email bookings.sssic@gmail.com, seats 520 (371 lower, 149 upper). Are these right, and is auditorium booking still offered?
+3. Social pages: facebook.com/SaiDelhiNCR and youtube.com/@SaidelhiOrg. Correct? Any Instagram or other official page?</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Text. Mark each line "correct" or give the new value.</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Have all from the old website and Google Maps (address: Bhisham Pitamah Marg, Pragati Vihar). Only question left: is there an Instagram or other official page?</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Hindi reviewer</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>A native Hindi speaker to read and correct the Hindi text on the website and in WhatsApp messages (written by us, not yet checked). Also the name of the group that reviews discourse translations, to credit on each discourse.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Name and WhatsApp number of the reviewer. They can mark changes in a shared document.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
           <t>Needed</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Seva figures (impact)</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Real yearly figures per programme for the Impact page, for example: medical camps held and people served, units of blood donated, eye surgeries, Bal Vikas children, Narayan Seva meals. The site currently shows sample numbers.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>One row per programme per year, with the source (report or register). Last 2 to 3 years if available.</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Totals only. No names of people helped.</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Old news posts only give per-event numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Partner list</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Hospitals, blood banks, trusts and NGOs we work with (for example ICARE Eye Hospital): name, type, city, and which programmes. Logos are row 5.</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Text list.</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Only partners who agree to be named.</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Old website mentions only ICARE Eye Hospital.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Home page pictures</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>1. Photo of the International Centre building, Lodhi Road (outside).
+2. Official centenary (100th birthday) artwork or logo, if one exists.
+3. Permission to use a still from the Sri Sathya Sai Answers YouTube channel, or a picture to show instead.</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Large original JPG, at least 1600 pixels wide. Logo as SVG or transparent PNG.</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Credit line for each. Centenary logo only with permission of its owner.</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>International Centre photo and centenary banner from the old website; Sai Answers picture from YouTube.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H8"/>
+  <autoFilter ref="A1:H14"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Needed,Requested,Received,Not needed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -892,7 +1203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -902,6 +1213,8 @@
     <col width="48" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -940,6 +1253,16 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Weekly gatherings</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Phone to show publicly</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
@@ -954,13 +1277,23 @@
       </c>
       <c r="C2" s="4" t="inlineStr"/>
       <c r="D2" s="4" t="inlineStr"/>
-      <c r="E2" s="4" t="inlineStr"/>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.572135,77.213929</t>
+        </is>
+      </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="n"/>
+      <c r="I2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -975,13 +1308,23 @@
       </c>
       <c r="C3" s="4" t="inlineStr"/>
       <c r="D3" s="4" t="inlineStr"/>
-      <c r="E3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.564903,77.240332</t>
+        </is>
+      </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -996,13 +1339,23 @@
       </c>
       <c r="C4" s="4" t="inlineStr"/>
       <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.574032,77.199067</t>
+        </is>
+      </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1017,13 +1370,23 @@
       </c>
       <c r="C5" s="4" t="inlineStr"/>
       <c r="D5" s="4" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.645507,77.228244</t>
+        </is>
+      </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -1038,13 +1401,23 @@
       </c>
       <c r="C6" s="4" t="inlineStr"/>
       <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.645605,77.212778</t>
+        </is>
+      </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -1078,6 +1451,8 @@
           <t>Prefilled from ssssoindia.org, please confirm</t>
         </is>
       </c>
+      <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -1108,9 +1483,11 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Prefilled from ssssoindia.org, please confirm</t>
-        </is>
-      </c>
+          <t>Two different pins: ssssoindia.org and the old website map are more than 1 km apart. Which is right?</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -1141,9 +1518,11 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Prefilled from ssssoindia.org, please confirm</t>
-        </is>
-      </c>
+          <t>Two different pins: ssssoindia.org and the old website map are more than 1 km apart. Which is right?</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -1158,13 +1537,23 @@
       </c>
       <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.612392,77.283974</t>
+        </is>
+      </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -1179,13 +1568,23 @@
       </c>
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.654882,77.305698</t>
+        </is>
+      </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -1200,13 +1599,23 @@
       </c>
       <c r="C12" s="4" t="inlineStr"/>
       <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.639425,77.310904</t>
+        </is>
+      </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -1221,13 +1630,23 @@
       </c>
       <c r="C13" s="4" t="inlineStr"/>
       <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.69897,77.138723</t>
+        </is>
+      </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="n"/>
+      <c r="I13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -1258,9 +1677,11 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Prefilled from ssssoindia.org, please confirm</t>
-        </is>
-      </c>
+          <t>Two different pins: ssssoindia.org and the old website map are more than 1 km apart. Which is right?</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -1275,13 +1696,23 @@
       </c>
       <c r="C15" s="4" t="inlineStr"/>
       <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.669126,77.092866</t>
+        </is>
+      </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="n"/>
+      <c r="I15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -1315,6 +1746,8 @@
           <t>Prefilled from ssssoindia.org, please confirm</t>
         </is>
       </c>
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -1329,13 +1762,23 @@
       </c>
       <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.690979,77.176524</t>
+        </is>
+      </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="n"/>
+      <c r="I17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -1369,6 +1812,8 @@
           <t>Prefilled from ssssoindia.org, please confirm</t>
         </is>
       </c>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
@@ -1383,13 +1828,23 @@
       </c>
       <c r="C19" s="4" t="inlineStr"/>
       <c r="D19" s="4" t="inlineStr"/>
-      <c r="E19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.539952,77.259158</t>
+        </is>
+      </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
@@ -1423,6 +1878,8 @@
           <t>Prefilled from ssssoindia.org, please confirm</t>
         </is>
       </c>
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
@@ -1437,13 +1894,23 @@
       </c>
       <c r="C21" s="4" t="inlineStr"/>
       <c r="D21" s="4" t="inlineStr"/>
-      <c r="E21" s="4" t="inlineStr"/>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.541506,77.216085</t>
+        </is>
+      </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
@@ -1458,13 +1925,23 @@
       </c>
       <c r="C22" s="4" t="inlineStr"/>
       <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="4" t="inlineStr"/>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.548202,77.238016</t>
+        </is>
+      </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
@@ -1479,13 +1956,23 @@
       </c>
       <c r="C23" s="4" t="inlineStr"/>
       <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.583419,77.168146</t>
+        </is>
+      </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="n"/>
+      <c r="I23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
@@ -1516,9 +2003,11 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Prefilled from ssssoindia.org, please confirm</t>
-        </is>
-      </c>
+          <t>Two different pins: ssssoindia.org and the old website map are more than 1 km apart. Which is right?</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="n"/>
+      <c r="I24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
@@ -1533,13 +2022,23 @@
       </c>
       <c r="C25" s="4" t="inlineStr"/>
       <c r="D25" s="4" t="inlineStr"/>
-      <c r="E25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.529312,77.148444</t>
+        </is>
+      </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="n"/>
+      <c r="I25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
@@ -1554,13 +2053,23 @@
       </c>
       <c r="C26" s="4" t="inlineStr"/>
       <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="4" t="inlineStr"/>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.558449,77.202938</t>
+        </is>
+      </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="n"/>
+      <c r="I26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
@@ -1575,13 +2084,23 @@
       </c>
       <c r="C27" s="4" t="inlineStr"/>
       <c r="D27" s="4" t="inlineStr"/>
-      <c r="E27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.534233,77.209447</t>
+        </is>
+      </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
@@ -1596,13 +2115,23 @@
       </c>
       <c r="C28" s="4" t="inlineStr"/>
       <c r="D28" s="4" t="inlineStr"/>
-      <c r="E28" s="4" t="inlineStr"/>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.638644,77.07206</t>
+        </is>
+      </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="n"/>
+      <c r="I28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
@@ -1617,13 +2146,23 @@
       </c>
       <c r="C29" s="4" t="inlineStr"/>
       <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.62486,77.110868</t>
+        </is>
+      </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="n"/>
+      <c r="I29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
@@ -1638,13 +2177,23 @@
       </c>
       <c r="C30" s="4" t="inlineStr"/>
       <c r="D30" s="4" t="inlineStr"/>
-      <c r="E30" s="4" t="inlineStr"/>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.649378,77.1437</t>
+        </is>
+      </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="n"/>
+      <c r="I30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
@@ -1675,9 +2224,11 @@
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Prefilled from ssssoindia.org, please confirm</t>
-        </is>
-      </c>
+          <t>Two different pins: ssssoindia.org and the old website map are more than 1 km apart. Which is right?</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="n"/>
+      <c r="I31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
@@ -1708,9 +2259,11 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Prefilled from ssssoindia.org, please confirm</t>
-        </is>
-      </c>
+          <t>Two different pins: ssssoindia.org and the old website map are more than 1 km apart. Which is right?</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="n"/>
+      <c r="I32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
@@ -1740,6 +2293,8 @@
           <t>Prefilled from ssssoindia.org, please confirm</t>
         </is>
       </c>
+      <c r="H33" s="4" t="n"/>
+      <c r="I33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
@@ -1752,15 +2307,29 @@
           <t>Faridabad 1</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Sector 7, 8, 9, 10 &amp; 11</t>
+        </is>
+      </c>
       <c r="D34" s="4" t="inlineStr"/>
-      <c r="E34" s="4" t="inlineStr"/>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.361738,77.326878</t>
+        </is>
+      </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="n"/>
+      <c r="I34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
@@ -1773,7 +2342,11 @@
           <t>Faridabad 3</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr"/>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Sector 14, 15, 16</t>
+        </is>
+      </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
           <t>457, Block A, ADB PWD Colony,  Sector 16 A, Faridabad, 121002</t>
@@ -1791,9 +2364,11 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Prefilled from ssssoindia.org, please confirm</t>
-        </is>
-      </c>
+          <t>Two different pins: ssssoindia.org and the old website map are more than 1 km apart. Which is right?</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="n"/>
+      <c r="I35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
@@ -1806,15 +2381,29 @@
           <t>Faridabad 5</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr"/>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Green Field, Charmwood</t>
+        </is>
+      </c>
       <c r="D36" s="4" t="inlineStr"/>
-      <c r="E36" s="4" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.458023,77.29641</t>
+        </is>
+      </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="n"/>
+      <c r="I36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
@@ -1835,7 +2424,13 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>No pin on the old website map</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="n"/>
+      <c r="I37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
@@ -1848,7 +2443,11 @@
           <t>Faridabad-2</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>NIT</t>
+        </is>
+      </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
           <t>B-33, Manglam Regency, Sector 21D, Near g b n school, Faridabad, 121012</t>
@@ -1866,9 +2465,11 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Prefilled from ssssoindia.org, please confirm</t>
-        </is>
-      </c>
+          <t>Two different pins: ssssoindia.org and the old website map are more than 1 km apart. Which is right?</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="n"/>
+      <c r="I38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
@@ -1881,7 +2482,11 @@
           <t>Faridabad-4</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr"/>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Sector 37, 91, IP Colony</t>
+        </is>
+      </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
           <t>530 sec 37, 1st floor, Faridabad, 121003</t>
@@ -1899,9 +2504,11 @@
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Prefilled from ssssoindia.org, please confirm</t>
-        </is>
-      </c>
+          <t>Two different pins: ssssoindia.org and the old website map are more than 1 km apart. Which is right?</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="n"/>
+      <c r="I39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
@@ -1914,15 +2521,29 @@
           <t>Gurugram 1</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr"/>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Laxman Vihar, Sector 4, 5, 7, 10, 37D, New Colony</t>
+        </is>
+      </c>
       <c r="D40" s="4" t="inlineStr"/>
-      <c r="E40" s="4" t="inlineStr"/>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.473804,77.010676</t>
+        </is>
+      </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="n"/>
+      <c r="I40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
@@ -1935,15 +2556,29 @@
           <t>Gurugram 2</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr"/>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>DLF 4, South City 1, Sector 31, 40, 45, 46, 50–57</t>
+        </is>
+      </c>
       <c r="D41" s="4" t="inlineStr"/>
-      <c r="E41" s="4" t="inlineStr"/>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.463441,77.076756</t>
+        </is>
+      </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="n"/>
+      <c r="I41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
@@ -1956,7 +2591,11 @@
           <t>Gurugram 3</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr"/>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>DLF Phase 1–5, Golf Course</t>
+        </is>
+      </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
           <t>7603, 2nd Floor, DLF Phase 4, Gurugram, 122009</t>
@@ -1974,9 +2613,11 @@
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Prefilled from ssssoindia.org, please confirm</t>
-        </is>
-      </c>
+          <t>Two different pins: ssssoindia.org and the old website map are more than 1 km apart. Which is right?</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="n"/>
+      <c r="I42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
@@ -1989,15 +2630,29 @@
           <t>Gurugram 4</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr"/>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Palam Vihar, Ashok Vihar, Brijwasan, Kapashera</t>
+        </is>
+      </c>
       <c r="D43" s="4" t="inlineStr"/>
-      <c r="E43" s="4" t="inlineStr"/>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.515197,77.035247</t>
+        </is>
+      </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="n"/>
+      <c r="I43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
@@ -2010,15 +2665,29 @@
           <t>Gurugram 5</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr"/>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Sohna Road, Rajiv Chowk to Badshahpur</t>
+        </is>
+      </c>
       <c r="D44" s="4" t="inlineStr"/>
-      <c r="E44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.433932,77.035701</t>
+        </is>
+      </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="n"/>
+      <c r="I44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
@@ -2031,15 +2700,29 @@
           <t>Gurugram 6</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr"/>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Sector 12–17</t>
+        </is>
+      </c>
       <c r="D45" s="4" t="inlineStr"/>
-      <c r="E45" s="4" t="inlineStr"/>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.471081,77.045414</t>
+        </is>
+      </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="n"/>
+      <c r="I45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
@@ -2052,15 +2735,29 @@
           <t>Gurugram 7 Samithi</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr"/>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Manesar, Sector 83–89</t>
+        </is>
+      </c>
       <c r="D46" s="4" t="inlineStr"/>
-      <c r="E46" s="4" t="inlineStr"/>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.40852,76.936938</t>
+        </is>
+      </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G46" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="n"/>
+      <c r="I46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
@@ -2075,13 +2772,23 @@
       </c>
       <c r="C47" s="4" t="inlineStr"/>
       <c r="D47" s="4" t="inlineStr"/>
-      <c r="E47" s="4" t="inlineStr"/>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.646018,77.369517</t>
+        </is>
+      </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="n"/>
+      <c r="I47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
@@ -2102,7 +2809,13 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="G48" s="4" t="inlineStr"/>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>No pin on the old website map</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="n"/>
+      <c r="I48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
@@ -2133,9 +2846,11 @@
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>Prefilled from ssssoindia.org, please confirm</t>
-        </is>
-      </c>
+          <t>Two different pins: ssssoindia.org and the old website map are more than 1 km apart. Which is right?</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="n"/>
+      <c r="I49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
@@ -2166,9 +2881,11 @@
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>Prefilled from ssssoindia.org, please confirm</t>
-        </is>
-      </c>
+          <t>Two different pins: ssssoindia.org and the old website map are more than 1 km apart. Which is right?</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="n"/>
+      <c r="I50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
@@ -2183,13 +2900,23 @@
       </c>
       <c r="C51" s="4" t="inlineStr"/>
       <c r="D51" s="4" t="inlineStr"/>
-      <c r="E51" s="4" t="inlineStr"/>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.504393,77.380432</t>
+        </is>
+      </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G51" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="n"/>
+      <c r="I51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
@@ -2210,7 +2937,13 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="G52" s="4" t="inlineStr"/>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>No pin on the old website map</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="n"/>
+      <c r="I52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
@@ -2244,6 +2977,8 @@
           <t>Prefilled from ssssoindia.org, please confirm</t>
         </is>
       </c>
+      <c r="H53" s="4" t="n"/>
+      <c r="I53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
@@ -2277,6 +3012,8 @@
           <t>Prefilled from ssssoindia.org, please confirm</t>
         </is>
       </c>
+      <c r="H54" s="4" t="n"/>
+      <c r="I54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
@@ -2307,9 +3044,11 @@
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>Prefilled from ssssoindia.org, please confirm</t>
-        </is>
-      </c>
+          <t>Two different pins: ssssoindia.org and the old website map are more than 1 km apart. Which is right?</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="n"/>
+      <c r="I55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
@@ -2324,13 +3063,23 @@
       </c>
       <c r="C56" s="4" t="inlineStr"/>
       <c r="D56" s="4" t="inlineStr"/>
-      <c r="E56" s="4" t="inlineStr"/>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.653564,77.460283</t>
+        </is>
+      </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G56" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="n"/>
+      <c r="I56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
@@ -2345,16 +3094,26 @@
       </c>
       <c r="C57" s="4" t="inlineStr"/>
       <c r="D57" s="4" t="inlineStr"/>
-      <c r="E57" s="4" t="inlineStr"/>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=28.819476,77.558411</t>
+        </is>
+      </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="G57" s="4" t="inlineStr"/>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>Pin from the old website map, please confirm; address and local name still needed</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="n"/>
+      <c r="I57" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G57"/>
+  <autoFilter ref="A1:I57"/>
   <dataValidations count="1">
     <dataValidation sqref="F2:F57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Needed,Requested,Received,Not needed"</formula1>

</xml_diff>